<commit_message>
chore: update MuleSoft job tracker
</commit_message>
<xml_diff>
--- a/MuleSoft_Job_Tracker.xlsx
+++ b/MuleSoft_Job_Tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet name="MuleSoft Jobs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MuleSoft Jobs'!$A$1:$F$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MuleSoft Jobs'!$A$1:$F$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -691,8 +691,40 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 12:24 IST</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise Integration | Anypoint Platform | Mulesoft</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise Integration | Anypoint Platform | Mulesoft</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>India / verify posting</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>47/100 — Matched profile skills: mulesoft, anypoint. Score 47/100.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>https://bing.com/ck/a</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F8"/>
+  <autoFilter ref="A1:F9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>